<commit_message>
Update: latest code changes
</commit_message>
<xml_diff>
--- a/outputs/filtered_profiles.xlsx
+++ b/outputs/filtered_profiles.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:AA2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,27 +491,27 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>pastJobTitle</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>liProfileImageUrl</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>isPremium</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>locationArea</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>connectionDegree</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>serviceProvider</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
@@ -568,24 +568,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gcc</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gcc</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/people/?keywords=Gcc</t>
+          <t>https://www.linkedin.com/search/results/people/?keywords=GCC</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>97748</v>
+        <v>99119</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -594,212 +594,93 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Baskar Kuppusamy</t>
+          <t>Abrar Shaikh</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Baskar</t>
+          <t>Abrar</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Kuppusamy</t>
+          <t>Shaikh</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>associate director | global capability center (gcc)</t>
+          <t>strategic talent acquisition &amp; sourcing. proven people-first approach and extensive experience in building high-performing teams. i gcc i ai in recruiting i ex - microsoft | johnson controls i spes i</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Associate Director | Global Capability Center (GCC)</t>
+          <t>Strategic Talent Acquisition &amp; sourcing. Proven People-First Approach and Extensive Experience in Building High-Performing Teams. I GCC I AI in recruiting I Ex - Microsoft | Johnson Controls I Spes I</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>https://media.licdn.com/dms/image/v2/C5603AQHcHXlXYvBi9Q/profile-displayphoto-shrink_100_100/profile-displayphoto-shrink_100_100/0/1668050454754?e=1756944000&amp;v=beta&amp;t=5483zB_ieXn2sxNGUPggNoa7O2TzZFvzqIUBATZiUH0</t>
-        </is>
-      </c>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
+          <t>https://media.licdn.com/dms/image/v2/D4D03AQGwdB9xbddaWw/profile-displayphoto-shrink_100_100/B4DZOcSFOeHcAY-/0/1733493807472?e=1757548800&amp;v=beta&amp;t=tSChqvCEpQUOw6LW1eorjIvbY3rj8v8nVf_GUG6P5jU</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>False</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Chennai</t>
-        </is>
-      </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>2nd degree connection</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ACoAAANQ_0gBFNd6M6YUt1Ss2uSYaq1pLoxGss8</t>
+          <t>https://www.linkedin.com/in/ACoAACWoH74BDGmmeXupJJg-FckWjYZ1c_Fse7I</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/baskar-kuppusamy-00877316</t>
+          <t>https://www.linkedin.com/in/abrar-shaikh-7666b6157</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>baskar-kuppusamy-00877316</t>
+          <t>abrar-shaikh-7666b6157</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/sales/people/ACoAAANQ_0gBFNd6M6YUt1Ss2uSYaq1pLoxGss8</t>
+          <t>https://www.linkedin.com/sales/people/ACoAACWoH74BDGmmeXupJJg-FckWjYZ1c_Fse7I</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>ACoAAANQ_0gBFNd6M6YUt1Ss2uSYaq1pLoxGss8</t>
+          <t>ACoAACWoH74BDGmmeXupJJg-FckWjYZ1c_Fse7I</t>
         </is>
       </c>
       <c r="W2" t="n">
-        <v>55639880</v>
+        <v>631775166</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>mdOmFPGbR/SmBxVWcVanhg==</t>
+          <t>soTLMK3XQuOh6W+E528zlA==</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/people/?facetNetwork=%22F%22&amp;facetConnectionOf=%22ACoAAANQ_0gBFNd6M6YUt1Ss2uSYaq1pLoxGss8%22&amp;origin=MEMBER_PROFILE_CANNED_SEARCH</t>
+          <t>https://www.linkedin.com/search/results/people/?facetNetwork=%22F%22&amp;facetConnectionOf=%22ACoAACWoH74BDGmmeXupJJg-FckWjYZ1c_Fse7I%22&amp;origin=MEMBER_PROFILE_CANNED_SEARCH</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2025-07-01T13:36:22.942Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Gcc</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Gcc</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/search/results/people/?keywords=Gcc</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" t="n">
-        <v>97748</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PEOPLE</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Siddharth (Sid) Dhandapani</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Siddharth</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>(Sid),Dhandapani</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>vice president &amp; head - gcc strategy and services</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Vice President &amp; Head - GCC Strategy and Services</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>https://media.licdn.com/dms/image/v2/D5635AQGBZST6WX2brg/profile-framedphoto-shrink_100_100/B56ZfB.XKeHEAo-/0/1751306040284?e=1751983200&amp;v=beta&amp;t=t0LTPARSFTSTTxzq4nwXfV5vbAx1i7hXslISVNyBQGY</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>3rd+ degree connection</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/ACoAAABl264BF13pWswV4yBJlLWAI90Qk6_KW0c</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/siddharth-sid-dhandapani-09229b2</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>siddharth-sid-dhandapani-09229b2</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/sales/people/ACoAAABl264BF13pWswV4yBJlLWAI90Qk6_KW0c</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>ACoAAABl264BF13pWswV4yBJlLWAI90Qk6_KW0c</t>
-        </is>
-      </c>
-      <c r="W3" t="n">
-        <v>6675374</v>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>6Sb91yYJRJqcN0n18uUa2Q==</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/search/results/people/?facetNetwork=%22F%22&amp;facetConnectionOf=%22ACoAAABl264BF13pWswV4yBJlLWAI90Qk6_KW0c%22&amp;origin=MEMBER_PROFILE_CANNED_SEARCH</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>2025-07-01T13:36:22.943Z</t>
+          <t>2025-07-09T11:07:37.951Z</t>
         </is>
       </c>
     </row>

</xml_diff>